<commit_message>
need to add status if its ready for accrual or not
</commit_message>
<xml_diff>
--- a/public/EXPORTING_FILE.xlsx
+++ b/public/EXPORTING_FILE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michael\Desktop\finall_scheduler\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A4A909D-605A-4CB1-85B6-6DD89C5D7909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55E5F06-F90D-4122-BDCA-86E471EC1AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,15 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId16" roundtripDataChecksum="97S5cfVxBL1/kpK/XWctiA8GK1Af71/O1vDD7Z4Kpi4="/>
     </ext>
@@ -365,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -401,24 +410,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -431,6 +427,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -440,11 +437,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -687,86 +699,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="28.5" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="23"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
+      <c r="Q1" s="19"/>
     </row>
     <row r="2" spans="1:27" ht="14.25" customHeight="1">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="23"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="19"/>
     </row>
     <row r="3" spans="1:27" ht="14.25" customHeight="1">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="32" t="s">
+      <c r="B3" s="22"/>
+      <c r="C3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="34" t="s">
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="35" t="s">
+      <c r="L3" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="M3" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="36"/>
-      <c r="O3" s="37"/>
-      <c r="P3" s="25" t="s">
+      <c r="N3" s="35"/>
+      <c r="O3" s="36"/>
+      <c r="P3" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="Q3" s="32" t="s">
+      <c r="Q3" s="25" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="49.5" customHeight="1">
-      <c r="A4" s="30"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="17"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="26"/>
       <c r="D4" s="1" t="s">
         <v>10</v>
       </c>
@@ -788,8 +800,8 @@
       <c r="J4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="31"/>
-      <c r="L4" s="17"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="26"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1" t="s">
         <v>15</v>
@@ -797,8 +809,8 @@
       <c r="O4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
     </row>
     <row r="5" spans="1:27" ht="49.5" hidden="1" customHeight="1">
       <c r="A5" s="5">
@@ -852,7 +864,7 @@
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="5"/>
-      <c r="D6" s="14"/>
+      <c r="D6" s="38"/>
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
       <c r="G6" s="14"/>
@@ -1467,148 +1479,148 @@
       <c r="AA25" s="12"/>
     </row>
     <row r="26" spans="1:27" ht="15.75" customHeight="1">
-      <c r="B26" s="18"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="19"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="19"/>
-      <c r="N26" s="19"/>
-      <c r="O26" s="19"/>
-      <c r="P26" s="19"/>
-      <c r="Q26" s="19"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="31"/>
+      <c r="M26" s="31"/>
+      <c r="N26" s="31"/>
+      <c r="O26" s="31"/>
+      <c r="P26" s="31"/>
+      <c r="Q26" s="31"/>
     </row>
     <row r="27" spans="1:27" ht="15.75" customHeight="1">
-      <c r="B27" s="20"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="21"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="21"/>
-      <c r="M27" s="21"/>
-      <c r="N27" s="21"/>
-      <c r="O27" s="21"/>
-      <c r="P27" s="21"/>
-      <c r="Q27" s="21"/>
+      <c r="B27" s="32"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="33"/>
+      <c r="J27" s="33"/>
+      <c r="K27" s="33"/>
+      <c r="L27" s="33"/>
+      <c r="M27" s="33"/>
+      <c r="N27" s="33"/>
+      <c r="O27" s="33"/>
+      <c r="P27" s="33"/>
+      <c r="Q27" s="33"/>
     </row>
     <row r="28" spans="1:27" ht="15.75" customHeight="1">
-      <c r="B28" s="20"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="21"/>
-      <c r="O28" s="21"/>
-      <c r="P28" s="21"/>
-      <c r="Q28" s="21"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
+      <c r="K28" s="33"/>
+      <c r="L28" s="33"/>
+      <c r="M28" s="33"/>
+      <c r="N28" s="33"/>
+      <c r="O28" s="33"/>
+      <c r="P28" s="33"/>
+      <c r="Q28" s="33"/>
     </row>
     <row r="29" spans="1:27" ht="15.75" customHeight="1">
-      <c r="B29" s="20"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="21"/>
-      <c r="I29" s="21"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="21"/>
-      <c r="L29" s="21"/>
-      <c r="M29" s="21"/>
-      <c r="N29" s="21"/>
-      <c r="O29" s="21"/>
-      <c r="P29" s="21"/>
-      <c r="Q29" s="21"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
+      <c r="K29" s="33"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="33"/>
+      <c r="N29" s="33"/>
+      <c r="O29" s="33"/>
+      <c r="P29" s="33"/>
+      <c r="Q29" s="33"/>
     </row>
     <row r="30" spans="1:27" ht="15.75" customHeight="1">
-      <c r="B30" s="20"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="21"/>
-      <c r="M30" s="21"/>
-      <c r="N30" s="21"/>
-      <c r="O30" s="21"/>
-      <c r="P30" s="21"/>
-      <c r="Q30" s="21"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="33"/>
+      <c r="N30" s="33"/>
+      <c r="O30" s="33"/>
+      <c r="P30" s="33"/>
+      <c r="Q30" s="33"/>
     </row>
     <row r="31" spans="1:27" ht="15.75" customHeight="1">
-      <c r="B31" s="20"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="21"/>
-      <c r="K31" s="21"/>
-      <c r="L31" s="21"/>
-      <c r="M31" s="21"/>
-      <c r="N31" s="21"/>
-      <c r="O31" s="21"/>
-      <c r="P31" s="21"/>
-      <c r="Q31" s="21"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="33"/>
+      <c r="J31" s="33"/>
+      <c r="K31" s="33"/>
+      <c r="L31" s="33"/>
+      <c r="M31" s="33"/>
+      <c r="N31" s="33"/>
+      <c r="O31" s="33"/>
+      <c r="P31" s="33"/>
+      <c r="Q31" s="33"/>
     </row>
     <row r="32" spans="1:27" ht="15.75" customHeight="1">
-      <c r="B32" s="20"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="21"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="21"/>
-      <c r="O32" s="21"/>
-      <c r="P32" s="21"/>
-      <c r="Q32" s="21"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="33"/>
+      <c r="J32" s="33"/>
+      <c r="K32" s="33"/>
+      <c r="L32" s="33"/>
+      <c r="M32" s="33"/>
+      <c r="N32" s="33"/>
+      <c r="O32" s="33"/>
+      <c r="P32" s="33"/>
+      <c r="Q32" s="33"/>
     </row>
     <row r="33" spans="2:17" ht="57.75" customHeight="1">
-      <c r="B33" s="20"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="21"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="21"/>
-      <c r="L33" s="21"/>
-      <c r="M33" s="21"/>
-      <c r="N33" s="21"/>
-      <c r="O33" s="21"/>
-      <c r="P33" s="21"/>
-      <c r="Q33" s="21"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+      <c r="G33" s="33"/>
+      <c r="H33" s="33"/>
+      <c r="I33" s="33"/>
+      <c r="J33" s="33"/>
+      <c r="K33" s="33"/>
+      <c r="L33" s="33"/>
+      <c r="M33" s="33"/>
+      <c r="N33" s="33"/>
+      <c r="O33" s="33"/>
+      <c r="P33" s="33"/>
+      <c r="Q33" s="33"/>
     </row>
     <row r="34" spans="2:17" ht="15.75" customHeight="1">
       <c r="P34" s="12"/>
@@ -2954,6 +2966,10 @@
     <row r="995" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B26:J33"/>
+    <mergeCell ref="K26:Q33"/>
+    <mergeCell ref="M3:O3"/>
+    <mergeCell ref="P3:P4"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A3:B4"/>
@@ -2962,10 +2978,6 @@
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="B26:J33"/>
-    <mergeCell ref="K26:Q33"/>
-    <mergeCell ref="M3:O3"/>
-    <mergeCell ref="P3:P4"/>
   </mergeCells>
   <pageMargins left="0.2" right="0.2" top="0.2" bottom="0.2" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape"/>

</xml_diff>